<commit_message>
Add quiz timer, result images, and audience updates
</commit_message>
<xml_diff>
--- a/public/quiz-template.xlsx
+++ b/public/quiz-template.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>#</t>
   </si>
@@ -50,7 +50,10 @@
     <t>Max score</t>
   </si>
   <si>
-    <t>animal type</t>
+    <t>Animal type</t>
+  </si>
+  <si>
+    <t>Image links</t>
   </si>
   <si>
     <t>Minimum</t>
@@ -77,7 +80,7 @@
     <t>Points: Choice 1 through Points: Choice 4 are numeric; a blank points cell counts as 0.</t>
   </si>
   <si>
-    <t>Max score, animal type, Minimum, Maximum, Description, and Recommendation are optional metadata.</t>
+    <t>Max score, Animal type, Image links, Minimum, Maximum, Description, and Recommendation are optional metadata.</t>
   </si>
   <si>
     <t>The # column is optional and is not used to identify questions.</t>
@@ -467,7 +470,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Q1"/>
+  <dimension ref="A1:R1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -476,11 +479,12 @@
     <col min="8" max="11" width="18" customWidth="1"/>
     <col min="12" max="12" width="14" customWidth="1"/>
     <col min="13" max="13" width="18" customWidth="1"/>
-    <col min="14" max="15" width="14" customWidth="1"/>
-    <col min="16" max="17" width="36" customWidth="1"/>
+    <col min="14" max="14" width="36" customWidth="1"/>
+    <col min="15" max="16" width="14" customWidth="1"/>
+    <col min="17" max="18" width="36" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -531,6 +535,9 @@
       </c>
       <c r="Q1" s="1" t="s">
         <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -549,32 +556,32 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>